<commit_message>
Update import reports for regenerated footer/adventures content
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures-listing.report.xlsx
+++ b/tools/importer/reports/import-adventures-listing.report.xlsx
@@ -67,7 +67,7 @@
     <t>footer</t>
   </si>
   <si>
-    <t>2026-09-23T08:09:25.089Z</t>
+    <t>2026-09-23T11:09:08.145Z</t>
   </si>
   <si>
     <t>WKND Footer</t>
@@ -82,7 +82,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-09-23T08:09:17.392Z</t>
+    <t>2026-09-23T09:22:55.096Z</t>
   </si>
   <si>
     <t>WKND Nav</t>
@@ -139,7 +139,7 @@
     <t>adventures-listing</t>
   </si>
   <si>
-    <t>2026-09-23T08:46:29.981Z</t>
+    <t>2026-09-23T11:18:24.871Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -196,7 +196,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-09-23T08:41:53.311Z</t>
+    <t>2026-09-23T08:46:34.482Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -211,7 +211,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-23T08:41:58.223Z</t>
+    <t>2026-09-23T08:46:38.545Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -226,7 +226,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:02.936Z</t>
+    <t>2026-09-23T08:46:43.939Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -241,7 +241,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:07.592Z</t>
+    <t>2026-09-23T08:46:49.566Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -256,7 +256,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:12.925Z</t>
+    <t>2026-09-23T08:46:53.656Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -271,7 +271,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:19.223Z</t>
+    <t>2026-09-23T08:46:57.963Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -286,7 +286,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:25.295Z</t>
+    <t>2026-09-23T08:47:02.548Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -301,7 +301,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:30.468Z</t>
+    <t>2026-09-23T08:47:07.436Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -316,7 +316,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:36.678Z</t>
+    <t>2026-09-23T08:47:13.832Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -331,7 +331,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:41.164Z</t>
+    <t>2026-09-23T08:47:19.473Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -346,7 +346,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:45.633Z</t>
+    <t>2026-09-23T08:47:25.177Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -361,7 +361,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:50.688Z</t>
+    <t>2026-09-23T08:47:30.307Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -376,7 +376,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-23T08:42:57.171Z</t>
+    <t>2026-09-23T08:47:36.666Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -391,7 +391,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-23T08:43:03.044Z</t>
+    <t>2026-09-23T08:47:41.750Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -406,7 +406,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-23T08:43:07.648Z</t>
+    <t>2026-09-23T08:47:46.981Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -421,7 +421,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-23T08:43:11.754Z</t>
+    <t>2026-09-23T08:47:52.497Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>

</xml_diff>